<commit_message>
Fixed hierarchy of The War / Osgiliath deeds
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-4-The War.xlsx
+++ b/_SourceFiles/DeedInfo-4-The War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\SourceFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE13E97-D59A-4D97-809C-3BC829E6B926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3065D476-8D49-42AC-8402-5325A9756135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5085" yWindow="1905" windowWidth="19995" windowHeight="10125" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3780" yWindow="1800" windowWidth="20115" windowHeight="12015" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -844,6 +844,7 @@
       <sheetName val="The Mountain-hold"/>
       <sheetName val="Return to Carn Dûm"/>
       <sheetName val="Corsairs of Umbar"/>
+      <sheetName val="The Legacy of Morgoth"/>
       <sheetName val="&lt;template&gt;"/>
     </sheetNames>
     <sheetDataSet>
@@ -1645,6 +1646,7 @@
       <sheetData sheetId="19"/>
       <sheetData sheetId="20"/>
       <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -10866,7 +10868,7 @@
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.42578125" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" customWidth="1"/>
+    <col min="11" max="11" width="55" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.140625" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
@@ -11150,22 +11152,22 @@
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>1879326410</v>
+        <v>1879326399</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
         <v>154</v>
       </c>
       <c r="G3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="K3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L3" t="s">
         <v>151</v>
@@ -11175,11 +11177,11 @@
       </c>
       <c r="R3" t="str">
         <f t="shared" ref="R3:R9" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
-        <v xml:space="preserve">  [2] = {["ID"] = 1879326410; }; -- Quest of the Court of Anárion -- Tier 1</v>
+        <v xml:space="preserve">  [2] = {["ID"] = 1879326399; }; -- Quest of the Court of Anárion -- Tier 3</v>
       </c>
       <c r="S3" s="1" t="str">
         <f t="shared" ref="S3:S9" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
-        <v xml:space="preserve">  [2] = {["ID"] = 1879326410; ["SAVE_INDEX"] = 2; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; };</v>
+        <v xml:space="preserve">  [2] = {["ID"] = 1879326399; ["SAVE_INDEX"] = 4; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; };</v>
       </c>
       <c r="T3">
         <f t="shared" ref="T3:T9" si="3">ROW()-1</f>
@@ -11191,11 +11193,11 @@
       </c>
       <c r="V3" t="str">
         <f t="shared" ref="V3:V9" si="5">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"                     ")</f>
-        <v xml:space="preserve">["ID"] = 1879326410; </v>
+        <v xml:space="preserve">["ID"] = 1879326399; </v>
       </c>
       <c r="W3" t="str">
         <f t="shared" ref="W3:W9" si="6">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
-        <v xml:space="preserve">["ID"] = 1879326410; </v>
+        <v xml:space="preserve">["ID"] = 1879326399; </v>
       </c>
       <c r="X3" t="str">
         <f t="shared" ref="X3:X9" si="7">IF(LEN(P3)&gt;0,CONCATENATE("[""CAT_ID""] = ",P3,"; "),"")</f>
@@ -11203,7 +11205,7 @@
       </c>
       <c r="Y3" s="1" t="str">
         <f t="shared" ref="Y3:Y9" si="8">IF(LEN(B3)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B3)),B3,"; "),REPT(" ",20))</f>
-        <v xml:space="preserve">["SAVE_INDEX"] = 2; </v>
+        <v xml:space="preserve">["SAVE_INDEX"] = 4; </v>
       </c>
       <c r="Z3">
         <f>VLOOKUP(D3,[1]Type!A$2:B$18,2,FALSE)</f>
@@ -11267,7 +11269,7 @@
       </c>
       <c r="AO3" t="str">
         <f t="shared" ref="AO3:AO9" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; </v>
       </c>
       <c r="AP3" t="str">
         <f t="shared" ref="AP3:AP9" si="22">CONCATENATE("[""LORE""] = { [""EN""] = """,L3,"""; }; ")</f>
@@ -11275,11 +11277,11 @@
       </c>
       <c r="AQ3" t="str">
         <f t="shared" ref="AQ3:AQ9" si="23">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K3,"""; }; ")</f>
-        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; </v>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; </v>
       </c>
       <c r="AR3" t="str">
         <f t="shared" ref="AR3:AR9" si="24">IF(LEN(G3)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G3,"""; }; "),"")</f>
-        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; </v>
+        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; </v>
       </c>
       <c r="AS3" t="str">
         <f t="shared" ref="AS3:AS9" si="25">CONCATENATE("};")</f>
@@ -11426,22 +11428,22 @@
     </row>
     <row r="5" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>1879326399</v>
+        <v>1879326410</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D5" t="s">
         <v>154</v>
       </c>
       <c r="G5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="K5" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="L5" t="s">
         <v>151</v>
@@ -11451,11 +11453,11 @@
       </c>
       <c r="R5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879326399; }; -- Quest of the Court of Anárion -- Tier 3</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; }; -- Quest of the Court of Anárion -- Tier 1</v>
       </c>
       <c r="S5" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879326399; ["SAVE_INDEX"] = 4; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; };</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; ["SAVE_INDEX"] = 2; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; };</v>
       </c>
       <c r="T5">
         <f t="shared" si="3"/>
@@ -11467,11 +11469,11 @@
       </c>
       <c r="V5" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["ID"] = 1879326399; </v>
+        <v xml:space="preserve">["ID"] = 1879326410; </v>
       </c>
       <c r="W5" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["ID"] = 1879326399; </v>
+        <v xml:space="preserve">["ID"] = 1879326410; </v>
       </c>
       <c r="X5" t="str">
         <f t="shared" si="7"/>
@@ -11479,7 +11481,7 @@
       </c>
       <c r="Y5" s="1" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">["SAVE_INDEX"] = 4; </v>
+        <v xml:space="preserve">["SAVE_INDEX"] = 2; </v>
       </c>
       <c r="Z5">
         <f>VLOOKUP(D5,[1]Type!A$2:B$18,2,FALSE)</f>
@@ -11543,7 +11545,7 @@
       </c>
       <c r="AO5" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; </v>
       </c>
       <c r="AP5" t="str">
         <f t="shared" si="22"/>
@@ -11551,11 +11553,11 @@
       </c>
       <c r="AQ5" t="str">
         <f t="shared" si="23"/>
-        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; </v>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; </v>
       </c>
       <c r="AR5" t="str">
         <f t="shared" si="24"/>
-        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; </v>
+        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; </v>
       </c>
       <c r="AS5" t="str">
         <f t="shared" si="25"/>
@@ -11564,22 +11566,22 @@
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>1879326404</v>
+        <v>1879326398</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
         <v>154</v>
       </c>
       <c r="G6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="K6" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="L6" t="s">
         <v>159</v>
@@ -11589,11 +11591,11 @@
       </c>
       <c r="R6" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [5] = {["ID"] = 1879326404; }; -- Quest of the Palace of Eldacar -- Tier 1</v>
+        <v xml:space="preserve">  [5] = {["ID"] = 1879326398; }; -- Quest of the Palace of Eldacar -- Tier 3</v>
       </c>
       <c r="S6" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [5] = {["ID"] = 1879326404; ["SAVE_INDEX"] = 5; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; };</v>
+        <v xml:space="preserve">  [5] = {["ID"] = 1879326398; ["SAVE_INDEX"] = 7; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; };</v>
       </c>
       <c r="T6">
         <f t="shared" si="3"/>
@@ -11605,11 +11607,11 @@
       </c>
       <c r="V6" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["ID"] = 1879326404; </v>
+        <v xml:space="preserve">["ID"] = 1879326398; </v>
       </c>
       <c r="W6" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["ID"] = 1879326404; </v>
+        <v xml:space="preserve">["ID"] = 1879326398; </v>
       </c>
       <c r="X6" t="str">
         <f t="shared" si="7"/>
@@ -11617,7 +11619,7 @@
       </c>
       <c r="Y6" s="1" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">["SAVE_INDEX"] = 5; </v>
+        <v xml:space="preserve">["SAVE_INDEX"] = 7; </v>
       </c>
       <c r="Z6">
         <f>VLOOKUP(D6,[1]Type!A$2:B$18,2,FALSE)</f>
@@ -11681,7 +11683,7 @@
       </c>
       <c r="AO6" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; </v>
       </c>
       <c r="AP6" t="str">
         <f t="shared" si="22"/>
@@ -11689,11 +11691,11 @@
       </c>
       <c r="AQ6" t="str">
         <f t="shared" si="23"/>
-        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; </v>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; </v>
       </c>
       <c r="AR6" t="str">
         <f t="shared" si="24"/>
-        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; </v>
+        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; </v>
       </c>
       <c r="AS6" t="str">
         <f t="shared" si="25"/>
@@ -11840,22 +11842,22 @@
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>1879326398</v>
+        <v>1879326404</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D8" t="s">
         <v>154</v>
       </c>
       <c r="G8" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="K8" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="L8" t="s">
         <v>159</v>
@@ -11865,11 +11867,11 @@
       </c>
       <c r="R8" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [7] = {["ID"] = 1879326398; }; -- Quest of the Palace of Eldacar -- Tier 3</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; }; -- Quest of the Palace of Eldacar -- Tier 1</v>
       </c>
       <c r="S8" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [7] = {["ID"] = 1879326398; ["SAVE_INDEX"] = 7; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; };</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; ["SAVE_INDEX"] = 5; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; };</v>
       </c>
       <c r="T8">
         <f t="shared" si="3"/>
@@ -11881,11 +11883,11 @@
       </c>
       <c r="V8" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["ID"] = 1879326398; </v>
+        <v xml:space="preserve">["ID"] = 1879326404; </v>
       </c>
       <c r="W8" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["ID"] = 1879326398; </v>
+        <v xml:space="preserve">["ID"] = 1879326404; </v>
       </c>
       <c r="X8" t="str">
         <f t="shared" si="7"/>
@@ -11893,7 +11895,7 @@
       </c>
       <c r="Y8" s="1" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">["SAVE_INDEX"] = 7; </v>
+        <v xml:space="preserve">["SAVE_INDEX"] = 5; </v>
       </c>
       <c r="Z8">
         <f>VLOOKUP(D8,[1]Type!A$2:B$18,2,FALSE)</f>
@@ -11957,7 +11959,7 @@
       </c>
       <c r="AO8" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; </v>
       </c>
       <c r="AP8" t="str">
         <f t="shared" si="22"/>
@@ -11965,11 +11967,11 @@
       </c>
       <c r="AQ8" t="str">
         <f t="shared" si="23"/>
-        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; </v>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; </v>
       </c>
       <c r="AR8" t="str">
         <f t="shared" si="24"/>
-        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; </v>
+        <v xml:space="preserve">["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; </v>
       </c>
       <c r="AS8" t="str">
         <f t="shared" si="25"/>
@@ -12281,8 +12283,9 @@
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:P8">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="14"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Encoded indents into DeedInfo.lua.
Fixed some incorrect indents as part of the process.
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-4-The War.xlsx
+++ b/_SourceFiles/DeedInfo-4-The War.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9B3A80-CB90-4BA2-B860-A8A0C987AEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46555C2D-EABC-4F92-A401-903613573BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23085" yWindow="2475" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19110" yWindow="1365" windowWidth="18600" windowHeight="14025" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -1935,9 +1935,10 @@
     <col min="3" max="3" width="34.42578125" customWidth="1"/>
     <col min="11" max="11" width="45.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.140625" customWidth="1"/>
+    <col min="18" max="18" width="29.85546875" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
     <col min="25" max="25" width="14" customWidth="1"/>
+    <col min="38" max="38" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.25">
@@ -2088,12 +2089,12 @@
         <v>120</v>
       </c>
       <c r="R2" t="str">
-        <f>CONCATENATE(U2,W2,X2,AS2," -- ",C2)</f>
+        <f>CONCATENATE(U2,W2,X2,AL2,AS2," -- ",C2)</f>
         <v xml:space="preserve">  [1] = {["CAT_ID"] = 120; }; -- Monster-slayer</v>
       </c>
       <c r="S2" s="1" t="str">
         <f>CONCATENATE(U2,V2,Y2,AA2,AC2,AE2,AG2,AI2,AK2,AL2,AM2,AN2,AO2,AP2,AQ2,AR2,AS2)</f>
-        <v xml:space="preserve">  [1] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Monster-slayer"; }; };</v>
+        <v xml:space="preserve">  [1] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Monster-slayer"; }; };</v>
       </c>
       <c r="T2">
         <f>ROW()-1</f>
@@ -2168,8 +2169,8 @@
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL2" t="str">
-        <f>CONCATENATE("[""TIER""] = ",TEXT(M2,"0"),"; ")</f>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <f>IF(M2&gt;0,CONCATENATE("[""TIER""] = ",TEXT(M2,"0"),"; "),"")</f>
+        <v/>
       </c>
       <c r="AM2" t="str">
         <f>IF(LEN(N2)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N2)),"""",N2,"""; "),"                    ")</f>
@@ -2229,12 +2230,12 @@
         <v>30</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R45" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
+        <f t="shared" ref="R3:R45" si="1">CONCATENATE(U3,W3,X3,AL3,AS3," -- ",C3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879071804; }; -- Monster-slayer -- Tier 7</v>
       </c>
       <c r="S3" s="1" t="str">
         <f t="shared" ref="S3:S46" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
-        <v xml:space="preserve">  [2] = {["ID"] = 1879071804; ["SAVE_INDEX"] =  1; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Monster-slayer -- Tier 7"; }; ["LORE"] = { ["EN"] = "Stem the tides of Darkness in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 50000 monster-players in the War"; }; ["TITLE"] = { ["EN"] = "Hero of Legend"; }; };</v>
+        <v xml:space="preserve">  [2] = {["ID"] = 1879071804; ["SAVE_INDEX"] =  1; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Monster-slayer -- Tier 7"; }; ["LORE"] = { ["EN"] = "Stem the tides of Darkness in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 50000 monster-players in the War"; }; ["TITLE"] = { ["EN"] = "Hero of Legend"; }; };</v>
       </c>
       <c r="T3">
         <f t="shared" ref="T3:T46" si="3">ROW()-1</f>
@@ -2309,8 +2310,8 @@
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL3" t="str">
-        <f t="shared" ref="AL3:AL46" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <f t="shared" ref="AL3:AL46" si="18">IF(M3&gt;0,CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; "),"")</f>
+        <v/>
       </c>
       <c r="AM3" t="str">
         <f t="shared" ref="AM3:AM46" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"                    ")</f>
@@ -2371,7 +2372,7 @@
       </c>
       <c r="R4" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [3] = {["ID"] = 1879071803; }; -- Monster-slayer -- Tier 6</v>
+        <v xml:space="preserve">  [3] = {["ID"] = 1879071803; ["TIER"] = 1; }; -- Monster-slayer -- Tier 6</v>
       </c>
       <c r="S4" s="1" t="str">
         <f t="shared" si="2"/>
@@ -2513,7 +2514,7 @@
       </c>
       <c r="R5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879071802; }; -- Monster-slayer -- Tier 5</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879071802; ["TIER"] = 2; }; -- Monster-slayer -- Tier 5</v>
       </c>
       <c r="S5" s="1" t="str">
         <f t="shared" si="2"/>
@@ -2654,7 +2655,7 @@
       </c>
       <c r="R6" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [5] = {["ID"] = 1879071801; }; -- Monster-slayer -- Tier 4</v>
+        <v xml:space="preserve">  [5] = {["ID"] = 1879071801; ["TIER"] = 3; }; -- Monster-slayer -- Tier 4</v>
       </c>
       <c r="S6" s="1" t="str">
         <f t="shared" si="2"/>
@@ -2795,7 +2796,7 @@
       </c>
       <c r="R7" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [6] = {["ID"] = 1879071800; }; -- Monster-slayer -- Tier 3</v>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879071800; ["TIER"] = 4; }; -- Monster-slayer -- Tier 3</v>
       </c>
       <c r="S7" s="1" t="str">
         <f t="shared" si="2"/>
@@ -2936,7 +2937,7 @@
       </c>
       <c r="R8" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [7] = {["ID"] = 1879071799; }; -- Monster-slayer -- Tier 2</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879071799; ["TIER"] = 5; }; -- Monster-slayer -- Tier 2</v>
       </c>
       <c r="S8" s="1" t="str">
         <f t="shared" si="2"/>
@@ -3077,7 +3078,7 @@
       </c>
       <c r="R9" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [8] = {["ID"] = 1879071798; }; -- Monster-slayer -- Tier 1</v>
+        <v xml:space="preserve">  [8] = {["ID"] = 1879071798; ["TIER"] = 6; }; -- Monster-slayer -- Tier 1</v>
       </c>
       <c r="S9" s="1" t="str">
         <f t="shared" si="2"/>
@@ -3204,7 +3205,7 @@
       </c>
       <c r="S10" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [9] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Blackarrow-slayer"; }; };</v>
+        <v xml:space="preserve">  [9] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Blackarrow-slayer"; }; };</v>
       </c>
       <c r="T10">
         <f t="shared" si="3"/>
@@ -3280,7 +3281,7 @@
       </c>
       <c r="AL10" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM10" t="str">
         <f t="shared" si="19"/>
@@ -3346,7 +3347,7 @@
       </c>
       <c r="S11" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [10] = {["ID"] = 1879071809; ["SAVE_INDEX"] =  8; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Blackarrow-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Uruk-blackarrows in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Uruk-blackarrows in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Blackarrow's Executioner"; }; };</v>
+        <v xml:space="preserve"> [10] = {["ID"] = 1879071809; ["SAVE_INDEX"] =  8; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Blackarrow-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Uruk-blackarrows in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Uruk-blackarrows in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Blackarrow's Executioner"; }; };</v>
       </c>
       <c r="T11">
         <f t="shared" si="3"/>
@@ -3422,7 +3423,7 @@
       </c>
       <c r="AL11" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM11" t="str">
         <f t="shared" si="19"/>
@@ -3483,7 +3484,7 @@
       </c>
       <c r="R12" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [11] = {["ID"] = 1879071808; }; -- Blackarrow-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [11] = {["ID"] = 1879071808; ["TIER"] = 1; }; -- Blackarrow-slayer -- Tier 4</v>
       </c>
       <c r="S12" s="1" t="str">
         <f t="shared" si="2"/>
@@ -3624,7 +3625,7 @@
       </c>
       <c r="R13" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [12] = {["ID"] = 1879071807; }; -- Blackarrow-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [12] = {["ID"] = 1879071807; ["TIER"] = 2; }; -- Blackarrow-slayer -- Tier 3</v>
       </c>
       <c r="S13" s="1" t="str">
         <f t="shared" si="2"/>
@@ -3765,7 +3766,7 @@
       </c>
       <c r="R14" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [13] = {["ID"] = 1879071806; }; -- Blackarrow-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [13] = {["ID"] = 1879071806; ["TIER"] = 3; }; -- Blackarrow-slayer -- Tier 2</v>
       </c>
       <c r="S14" s="1" t="str">
         <f t="shared" si="2"/>
@@ -3906,7 +3907,7 @@
       </c>
       <c r="R15" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [14] = {["ID"] = 1879071805; }; -- Blackarrow-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [14] = {["ID"] = 1879071805; ["TIER"] = 4; }; -- Blackarrow-slayer -- Tier 1</v>
       </c>
       <c r="S15" s="1" t="str">
         <f t="shared" si="2"/>
@@ -4033,7 +4034,7 @@
       </c>
       <c r="S16" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [15] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Reaver-slayer"; }; };</v>
+        <v xml:space="preserve"> [15] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Reaver-slayer"; }; };</v>
       </c>
       <c r="T16">
         <f t="shared" si="3"/>
@@ -4109,7 +4110,7 @@
       </c>
       <c r="AL16" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM16" t="str">
         <f t="shared" si="19"/>
@@ -4175,7 +4176,7 @@
       </c>
       <c r="S17" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [16] = {["ID"] = 1879071814; ["SAVE_INDEX"] = 13; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Reaver-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Orc-reavers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Reavers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Reaver's End"; }; };</v>
+        <v xml:space="preserve"> [16] = {["ID"] = 1879071814; ["SAVE_INDEX"] = 13; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Reaver-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Orc-reavers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Reavers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Reaver's End"; }; };</v>
       </c>
       <c r="T17">
         <f t="shared" si="3"/>
@@ -4251,7 +4252,7 @@
       </c>
       <c r="AL17" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM17" t="str">
         <f t="shared" si="19"/>
@@ -4312,7 +4313,7 @@
       </c>
       <c r="R18" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [17] = {["ID"] = 1879071813; }; -- Reaver-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [17] = {["ID"] = 1879071813; ["TIER"] = 1; }; -- Reaver-slayer -- Tier 4</v>
       </c>
       <c r="S18" s="1" t="str">
         <f t="shared" si="2"/>
@@ -4453,7 +4454,7 @@
       </c>
       <c r="R19" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [18] = {["ID"] = 1879071812; }; -- Reaver-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [18] = {["ID"] = 1879071812; ["TIER"] = 2; }; -- Reaver-slayer -- Tier 3</v>
       </c>
       <c r="S19" s="1" t="str">
         <f t="shared" si="2"/>
@@ -4594,7 +4595,7 @@
       </c>
       <c r="R20" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [19] = {["ID"] = 1879071811; }; -- Reaver-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [19] = {["ID"] = 1879071811; ["TIER"] = 3; }; -- Reaver-slayer -- Tier 2</v>
       </c>
       <c r="S20" s="1" t="str">
         <f t="shared" si="2"/>
@@ -4735,7 +4736,7 @@
       </c>
       <c r="R21" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [20] = {["ID"] = 1879071810; }; -- Reaver-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [20] = {["ID"] = 1879071810; ["TIER"] = 4; }; -- Reaver-slayer -- Tier 1</v>
       </c>
       <c r="S21" s="1" t="str">
         <f t="shared" si="2"/>
@@ -4862,7 +4863,7 @@
       </c>
       <c r="S22" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [21] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Defiler-slayer"; }; };</v>
+        <v xml:space="preserve"> [21] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Defiler-slayer"; }; };</v>
       </c>
       <c r="T22">
         <f t="shared" si="3"/>
@@ -4938,7 +4939,7 @@
       </c>
       <c r="AL22" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM22" t="str">
         <f t="shared" si="19"/>
@@ -5003,7 +5004,7 @@
       </c>
       <c r="S23" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [22] = {["ID"] = 1879071819; ["SAVE_INDEX"] = 18; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Defiler-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Orc-defilers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Defilers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Weird of the Defilers"; }; };</v>
+        <v xml:space="preserve"> [22] = {["ID"] = 1879071819; ["SAVE_INDEX"] = 18; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Defiler-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Orc-defilers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Defilers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Weird of the Defilers"; }; };</v>
       </c>
       <c r="T23">
         <f t="shared" si="3"/>
@@ -5079,7 +5080,7 @@
       </c>
       <c r="AL23" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM23" t="str">
         <f t="shared" si="19"/>
@@ -5140,7 +5141,7 @@
       </c>
       <c r="R24" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [23] = {["ID"] = 1879071818; }; -- Defiler-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [23] = {["ID"] = 1879071818; ["TIER"] = 1; }; -- Defiler-slayer -- Tier 4</v>
       </c>
       <c r="S24" s="1" t="str">
         <f t="shared" si="2"/>
@@ -5281,7 +5282,7 @@
       </c>
       <c r="R25" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [24] = {["ID"] = 1879071817; }; -- Defiler-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [24] = {["ID"] = 1879071817; ["TIER"] = 2; }; -- Defiler-slayer -- Tier 3</v>
       </c>
       <c r="S25" s="1" t="str">
         <f t="shared" si="2"/>
@@ -5423,7 +5424,7 @@
       </c>
       <c r="R26" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [25] = {["ID"] = 1879071816; }; -- Defiler-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [25] = {["ID"] = 1879071816; ["TIER"] = 3; }; -- Defiler-slayer -- Tier 2</v>
       </c>
       <c r="S26" s="1" t="str">
         <f t="shared" si="2"/>
@@ -5564,7 +5565,7 @@
       </c>
       <c r="R27" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [26] = {["ID"] = 1879071815; }; -- Defiler-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [26] = {["ID"] = 1879071815; ["TIER"] = 4; }; -- Defiler-slayer -- Tier 1</v>
       </c>
       <c r="S27" s="1" t="str">
         <f t="shared" si="2"/>
@@ -5691,7 +5692,7 @@
       </c>
       <c r="S28" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [27] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Stalker-slayer"; }; };</v>
+        <v xml:space="preserve"> [27] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Stalker-slayer"; }; };</v>
       </c>
       <c r="T28">
         <f t="shared" si="3"/>
@@ -5767,7 +5768,7 @@
       </c>
       <c r="AL28" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM28" t="str">
         <f t="shared" si="19"/>
@@ -5832,7 +5833,7 @@
       </c>
       <c r="S29" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [28] = {["ID"] = 1879071824; ["SAVE_INDEX"] = 23; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Stalker-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Warg-stalkers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Stalkers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Stalker's Nemesis"; }; };</v>
+        <v xml:space="preserve"> [28] = {["ID"] = 1879071824; ["SAVE_INDEX"] = 23; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Stalker-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Warg-stalkers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Stalkers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Stalker's Nemesis"; }; };</v>
       </c>
       <c r="T29">
         <f t="shared" si="3"/>
@@ -5908,7 +5909,7 @@
       </c>
       <c r="AL29" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM29" t="str">
         <f t="shared" si="19"/>
@@ -5969,7 +5970,7 @@
       </c>
       <c r="R30" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [29] = {["ID"] = 1879071823; }; -- Stalker-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [29] = {["ID"] = 1879071823; ["TIER"] = 1; }; -- Stalker-slayer -- Tier 4</v>
       </c>
       <c r="S30" s="1" t="str">
         <f t="shared" si="2"/>
@@ -6110,7 +6111,7 @@
       </c>
       <c r="R31" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [30] = {["ID"] = 1879071822; }; -- Stalker-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [30] = {["ID"] = 1879071822; ["TIER"] = 2; }; -- Stalker-slayer -- Tier 3</v>
       </c>
       <c r="S31" s="1" t="str">
         <f t="shared" si="2"/>
@@ -6252,7 +6253,7 @@
       </c>
       <c r="R32" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [31] = {["ID"] = 1879071821; }; -- Stalker-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [31] = {["ID"] = 1879071821; ["TIER"] = 3; }; -- Stalker-slayer -- Tier 2</v>
       </c>
       <c r="S32" s="1" t="str">
         <f t="shared" si="2"/>
@@ -6393,7 +6394,7 @@
       </c>
       <c r="R33" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [32] = {["ID"] = 1879071820; }; -- Stalker-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [32] = {["ID"] = 1879071820; ["TIER"] = 4; }; -- Stalker-slayer -- Tier 1</v>
       </c>
       <c r="S33" s="1" t="str">
         <f t="shared" si="2"/>
@@ -6520,7 +6521,7 @@
       </c>
       <c r="S34" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [33] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Warleader-slayer"; }; };</v>
+        <v xml:space="preserve"> [33] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Warleader-slayer"; }; };</v>
       </c>
       <c r="T34">
         <f t="shared" si="3"/>
@@ -6596,7 +6597,7 @@
       </c>
       <c r="AL34" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM34" t="str">
         <f t="shared" si="19"/>
@@ -6661,7 +6662,7 @@
       </c>
       <c r="S35" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [34] = {["ID"] = 1879071829; ["SAVE_INDEX"] = 28; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Warleader-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Uruk-warleaders in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Warleaders in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "War-leader's Doom"; }; };</v>
+        <v xml:space="preserve"> [34] = {["ID"] = 1879071829; ["SAVE_INDEX"] = 28; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Warleader-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Uruk-warleaders in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Warleaders in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "War-leader's Doom"; }; };</v>
       </c>
       <c r="T35">
         <f t="shared" si="3"/>
@@ -6737,7 +6738,7 @@
       </c>
       <c r="AL35" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM35" t="str">
         <f t="shared" si="19"/>
@@ -6798,7 +6799,7 @@
       </c>
       <c r="R36" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [35] = {["ID"] = 1879071828; }; -- Warleader-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [35] = {["ID"] = 1879071828; ["TIER"] = 1; }; -- Warleader-slayer -- Tier 4</v>
       </c>
       <c r="S36" s="1" t="str">
         <f t="shared" si="2"/>
@@ -6939,7 +6940,7 @@
       </c>
       <c r="R37" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [36] = {["ID"] = 1879071827; }; -- Warleader-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [36] = {["ID"] = 1879071827; ["TIER"] = 2; }; -- Warleader-slayer -- Tier 3</v>
       </c>
       <c r="S37" s="1" t="str">
         <f t="shared" si="2"/>
@@ -7080,7 +7081,7 @@
       </c>
       <c r="R38" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [37] = {["ID"] = 1879071826; }; -- Warleader-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [37] = {["ID"] = 1879071826; ["TIER"] = 3; }; -- Warleader-slayer -- Tier 2</v>
       </c>
       <c r="S38" s="1" t="str">
         <f t="shared" si="2"/>
@@ -7221,7 +7222,7 @@
       </c>
       <c r="R39" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [38] = {["ID"] = 1879071825; }; -- Warleader-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [38] = {["ID"] = 1879071825; ["TIER"] = 4; }; -- Warleader-slayer -- Tier 1</v>
       </c>
       <c r="S39" s="1" t="str">
         <f t="shared" si="2"/>
@@ -7348,7 +7349,7 @@
       </c>
       <c r="S40" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [39] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0;                     ["NAME"] = { ["EN"] = "Weaver-slayer"; }; };</v>
+        <v xml:space="preserve"> [39] = {                                          ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1;                     ["NAME"] = { ["EN"] = "Weaver-slayer"; }; };</v>
       </c>
       <c r="T40">
         <f t="shared" si="3"/>
@@ -7424,7 +7425,7 @@
       </c>
       <c r="AL40" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM40" t="str">
         <f t="shared" si="19"/>
@@ -7489,7 +7490,7 @@
       </c>
       <c r="S41" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [40] = {["ID"] = 1879071834; ["SAVE_INDEX"] = 33; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Weaver-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Weavers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Weavers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Exterminator of Weavers"; }; };</v>
+        <v xml:space="preserve"> [40] = {["ID"] = 1879071834; ["SAVE_INDEX"] = 33; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "30"; ["NAME"] = { ["EN"] = "Weaver-slayer -- Tier 5"; }; ["LORE"] = { ["EN"] = "Stem the tide of Weavers in the War."; }; ["SUMMARY"] = { ["EN"] = "Defeat 10000 Weavers in the Ettenmoors"; }; ["TITLE"] = { ["EN"] = "Exterminator of Weavers"; }; };</v>
       </c>
       <c r="T41">
         <f t="shared" si="3"/>
@@ -7565,7 +7566,7 @@
       </c>
       <c r="AL41" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM41" t="str">
         <f t="shared" si="19"/>
@@ -7626,7 +7627,7 @@
       </c>
       <c r="R42" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [41] = {["ID"] = 1879071833; }; -- Weaver-slayer -- Tier 4</v>
+        <v xml:space="preserve"> [41] = {["ID"] = 1879071833; ["TIER"] = 1; }; -- Weaver-slayer -- Tier 4</v>
       </c>
       <c r="S42" s="1" t="str">
         <f t="shared" si="2"/>
@@ -7767,7 +7768,7 @@
       </c>
       <c r="R43" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [42] = {["ID"] = 1879071832; }; -- Weaver-slayer -- Tier 3</v>
+        <v xml:space="preserve"> [42] = {["ID"] = 1879071832; ["TIER"] = 2; }; -- Weaver-slayer -- Tier 3</v>
       </c>
       <c r="S43" s="1" t="str">
         <f t="shared" si="2"/>
@@ -7908,7 +7909,7 @@
       </c>
       <c r="R44" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [43] = {["ID"] = 1879071831; }; -- Weaver-slayer -- Tier 2</v>
+        <v xml:space="preserve"> [43] = {["ID"] = 1879071831; ["TIER"] = 3; }; -- Weaver-slayer -- Tier 2</v>
       </c>
       <c r="S44" s="1" t="str">
         <f t="shared" si="2"/>
@@ -8049,7 +8050,7 @@
       </c>
       <c r="R45" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [44] = {["ID"] = 1879071830; }; -- Weaver-slayer -- Tier 1</v>
+        <v xml:space="preserve"> [44] = {["ID"] = 1879071830; ["TIER"] = 4; }; -- Weaver-slayer -- Tier 1</v>
       </c>
       <c r="S45" s="1" t="str">
         <f t="shared" si="2"/>
@@ -8239,7 +8240,7 @@
       </c>
       <c r="AL46" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM46" t="str">
         <f t="shared" si="19"/>
@@ -8281,6 +8282,7 @@
     <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10995,9 +10997,10 @@
     <col min="3" max="3" width="34.42578125" customWidth="1"/>
     <col min="11" max="11" width="55" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.140625" customWidth="1"/>
+    <col min="18" max="18" width="31.42578125" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
     <col min="25" max="25" width="14" customWidth="1"/>
+    <col min="38" max="38" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.25">
@@ -11163,12 +11166,12 @@
         <v>90</v>
       </c>
       <c r="R2" t="str">
-        <f>CONCATENATE(U2,W2,X2,AS2," -- ",C2)</f>
+        <f>CONCATENATE(U2,W2,X2,AL2,AS2," -- ",C2)</f>
         <v xml:space="preserve">  [1] = {["ID"] = 1879326392; }; -- The Battle for Osgiliath</v>
       </c>
       <c r="S2" s="1" t="str">
         <f>CONCATENATE(U2,V2,Y2,AA2,AC2,AE2,AG2,AI2,AK2,AL2,AM2,AN2,AO2,AP2,AQ2,AR2,AS2)</f>
-        <v xml:space="preserve">  [1] = {["ID"] = 1879326392; ["SAVE_INDEX"] = 1; ["TYPE"] = 3; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "90"; ["NAME"] = { ["EN"] = "The Battle for Osgiliath"; }; ["LORE"] = { ["EN"] = "Explore the battleground of Osgiliath."; }; ["SUMMARY"] = { ["EN"] = "Discover 7 locations"; }; ["TITLE"] = { ["EN"] = "Surveyor of Battle"; }; };</v>
+        <v xml:space="preserve">  [1] = {["ID"] = 1879326392; ["SAVE_INDEX"] = 1; ["TYPE"] = 3; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "90"; ["NAME"] = { ["EN"] = "The Battle for Osgiliath"; }; ["LORE"] = { ["EN"] = "Explore the battleground of Osgiliath."; }; ["SUMMARY"] = { ["EN"] = "Discover 7 locations"; }; ["TITLE"] = { ["EN"] = "Surveyor of Battle"; }; };</v>
       </c>
       <c r="T2">
         <f>ROW()-1</f>
@@ -11243,8 +11246,8 @@
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL2" t="str">
-        <f>CONCATENATE("[""TIER""] = ",TEXT(M2,"0"),"; ")</f>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <f>IF(M2&gt;0,CONCATENATE("[""TIER""] = ",TEXT(M2,"0"),"; "),"")</f>
+        <v/>
       </c>
       <c r="AM2" t="str">
         <f>IF(LEN(N2)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N2)),"""",N2,"""; "),"")</f>
@@ -11301,12 +11304,12 @@
         <v>50</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R9" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
+        <f t="shared" ref="R3:R9" si="1">CONCATENATE(U3,W3,X3,AL3,AS3," -- ",C3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879326399; }; -- Quest of the Court of Anárion -- Tier 3</v>
       </c>
       <c r="S3" s="1" t="str">
         <f t="shared" ref="S3:S9" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
-        <v xml:space="preserve">  [2] = {["ID"] = 1879326399; ["SAVE_INDEX"] = 4; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; };</v>
+        <v xml:space="preserve">  [2] = {["ID"] = 1879326399; ["SAVE_INDEX"] = 4; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 50 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Warrior"; }; };</v>
       </c>
       <c r="T3">
         <f t="shared" ref="T3:T9" si="3">ROW()-1</f>
@@ -11381,8 +11384,8 @@
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL3" t="str">
-        <f t="shared" ref="AL3:AL9" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <f t="shared" ref="AL3:AL9" si="18">IF(M3&gt;0,CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; "),"")</f>
+        <v/>
       </c>
       <c r="AM3" t="str">
         <f t="shared" ref="AM3:AM9" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"")</f>
@@ -11435,16 +11438,19 @@
       <c r="L4" t="s">
         <v>151</v>
       </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
       <c r="N4">
         <v>50</v>
       </c>
       <c r="R4" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [3] = {["ID"] = 1879326396; }; -- Quest of the Court of Anárion -- Tier 2</v>
+        <v xml:space="preserve">  [3] = {["ID"] = 1879326396; ["TIER"] = 1; }; -- Quest of the Court of Anárion -- Tier 2</v>
       </c>
       <c r="S4" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [3] = {["ID"] = 1879326396; ["SAVE_INDEX"] = 3; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 2"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 25 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Soldier"; }; };</v>
+        <v xml:space="preserve">  [3] = {["ID"] = 1879326396; ["SAVE_INDEX"] = 3; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 1; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 2"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 25 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Soldier"; }; };</v>
       </c>
       <c r="T4">
         <f t="shared" si="3"/>
@@ -11520,7 +11526,7 @@
       </c>
       <c r="AL4" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AM4" t="str">
         <f t="shared" si="19"/>
@@ -11573,16 +11579,19 @@
       <c r="L5" t="s">
         <v>151</v>
       </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
       <c r="N5">
         <v>50</v>
       </c>
       <c r="R5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; }; -- Quest of the Court of Anárion -- Tier 1</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; ["TIER"] = 2; }; -- Quest of the Court of Anárion -- Tier 1</v>
       </c>
       <c r="S5" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; ["SAVE_INDEX"] = 2; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; };</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879326410; ["SAVE_INDEX"] = 2; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 2; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Court of Anárion -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captain of the Court of Anárion will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 10 quests for the benefit of the Court of Anárion!"; }; ["TITLE"] = { ["EN"] = "Gondorian Recruit"; }; };</v>
       </c>
       <c r="T5">
         <f t="shared" si="3"/>
@@ -11658,7 +11667,7 @@
       </c>
       <c r="AL5" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="AM5" t="str">
         <f t="shared" si="19"/>
@@ -11720,7 +11729,7 @@
       </c>
       <c r="S6" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [5] = {["ID"] = 1879326398; ["SAVE_INDEX"] = 7; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; };</v>
+        <v xml:space="preserve">  [5] = {["ID"] = 1879326398; ["SAVE_INDEX"] = 7; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 3"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 80 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Shield of Eldacar"; }; };</v>
       </c>
       <c r="T6">
         <f t="shared" si="3"/>
@@ -11796,7 +11805,7 @@
       </c>
       <c r="AL6" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM6" t="str">
         <f t="shared" si="19"/>
@@ -11849,16 +11858,19 @@
       <c r="L7" t="s">
         <v>159</v>
       </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
       <c r="N7">
         <v>50</v>
       </c>
       <c r="R7" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [6] = {["ID"] = 1879326401; }; -- Quest of the Palace of Eldacar -- Tier 2</v>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879326401; ["TIER"] = 1; }; -- Quest of the Palace of Eldacar -- Tier 2</v>
       </c>
       <c r="S7" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [6] = {["ID"] = 1879326401; ["SAVE_INDEX"] = 6; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 2"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 40 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Protector of Eldacar"; }; };</v>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879326401; ["SAVE_INDEX"] = 6; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 1; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 2"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 40 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Protector of Eldacar"; }; };</v>
       </c>
       <c r="T7">
         <f t="shared" si="3"/>
@@ -11934,7 +11946,7 @@
       </c>
       <c r="AL7" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="AM7" t="str">
         <f t="shared" si="19"/>
@@ -11987,16 +11999,19 @@
       <c r="L8" t="s">
         <v>159</v>
       </c>
+      <c r="M8">
+        <v>2</v>
+      </c>
       <c r="N8">
         <v>50</v>
       </c>
       <c r="R8" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; }; -- Quest of the Palace of Eldacar -- Tier 1</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; ["TIER"] = 2; }; -- Quest of the Palace of Eldacar -- Tier 1</v>
       </c>
       <c r="S8" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; ["SAVE_INDEX"] = 5; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; };</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879326404; ["SAVE_INDEX"] = 5; ["TYPE"] = 7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 2; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Quest of the Palace of Eldacar -- Tier 1"; }; ["LORE"] = { ["EN"] = "Service to the captains of the Palace of Eldacar will result in the ability to find your way through the city with less effort."; }; ["SUMMARY"] = { ["EN"] = "Complete 15 quests for the benefit of the Palace of Eldacar!"; }; ["TITLE"] = { ["EN"] = "Defender of Eldacar"; }; };</v>
       </c>
       <c r="T8">
         <f t="shared" si="3"/>
@@ -12072,7 +12087,7 @@
       </c>
       <c r="AL8" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="AM8" t="str">
         <f t="shared" si="19"/>
@@ -12186,7 +12201,7 @@
       </c>
       <c r="AL9" t="str">
         <f t="shared" si="18"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v/>
       </c>
       <c r="AM9" t="str">
         <f t="shared" si="19"/>
@@ -12411,6 +12426,6 @@
     <cfRule type="duplicateValues" dxfId="0" priority="14"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated The War category names with season numbers.
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-4-The War.xlsx
+++ b/_SourceFiles/DeedInfo-4-The War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689AA7FF-03F4-4D57-96A6-0FA5B8F044A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD345887-F509-4311-A102-B64DB99E36BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8205" yWindow="5415" windowWidth="20895" windowHeight="10320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -635,33 +635,18 @@
     <t>Title: Preserver of Order</t>
   </si>
   <si>
-    <t>- Monster Player Reward Season 1 -</t>
-  </si>
-  <si>
     <t>Title: Exemplar</t>
   </si>
   <si>
     <t>Limited Time Only</t>
   </si>
   <si>
-    <t>- Season of the Nemesis -</t>
-  </si>
-  <si>
     <t>Title: Benevolence Incarnate</t>
   </si>
   <si>
     <t>Title: The Respected Voice</t>
   </si>
   <si>
-    <t>- Season of Scorn -</t>
-  </si>
-  <si>
-    <t>- Season of Spirit -</t>
-  </si>
-  <si>
-    <t>- Season of Malice -</t>
-  </si>
-  <si>
     <t>Title: The Spirit's Guide</t>
   </si>
   <si>
@@ -671,7 +656,22 @@
     <t>Title: Bastion of Light</t>
   </si>
   <si>
-    <t>- Monster Player Reward Season 6 -</t>
+    <t>- Season 1: Strife -</t>
+  </si>
+  <si>
+    <t>- Season 2: Nemesis -</t>
+  </si>
+  <si>
+    <t>- Season 3: Malice -</t>
+  </si>
+  <si>
+    <t>- Season 4: Scorn -</t>
+  </si>
+  <si>
+    <t>- Season 5: Spirits -</t>
+  </si>
+  <si>
+    <t>- Season 6: Rivals -</t>
   </si>
 </sst>
 </file>
@@ -721,11 +721,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -8615,11 +8614,11 @@
         <v>50</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R22" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
+        <f t="shared" ref="R3:R18" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879071836; }; -- Conquest of Dargazag</v>
       </c>
       <c r="S3" s="1" t="str">
-        <f t="shared" ref="S3:S22" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
+        <f t="shared" ref="S3:S18" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879071836; ["SAVE_INDEX"] = 2; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; ["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; };</v>
       </c>
       <c r="T3">
@@ -8627,23 +8626,23 @@
         <v>2</v>
       </c>
       <c r="U3" t="str">
-        <f t="shared" ref="U3:U22" si="4">CONCATENATE(REPT(" ",3-LEN(T3)),"[",T3,"] = {")</f>
+        <f t="shared" ref="U3:U18" si="4">CONCATENATE(REPT(" ",3-LEN(T3)),"[",T3,"] = {")</f>
         <v xml:space="preserve">  [2] = {</v>
       </c>
       <c r="V3" t="str">
-        <f t="shared" ref="V3:V22" si="5">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"                     ")</f>
+        <f t="shared" ref="V3:V18" si="5">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"                     ")</f>
         <v xml:space="preserve">["ID"] = 1879071836; </v>
       </c>
       <c r="W3" t="str">
-        <f t="shared" ref="W3:W22" si="6">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
+        <f t="shared" ref="W3:W18" si="6">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879071836; </v>
       </c>
       <c r="X3" t="str">
-        <f t="shared" ref="X3:X22" si="7">IF(LEN(P3)&gt;0,CONCATENATE("[""CAT_ID""] = ",P3,"; "),"")</f>
+        <f t="shared" ref="X3:X18" si="7">IF(LEN(P3)&gt;0,CONCATENATE("[""CAT_ID""] = ",P3,"; "),"")</f>
         <v/>
       </c>
       <c r="Y3" s="1" t="str">
-        <f t="shared" ref="Y3:Y22" si="8">IF(LEN(B3)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B3)),B3,"; "),REPT(" ",20))</f>
+        <f t="shared" ref="Y3:Y18" si="8">IF(LEN(B3)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B3)),B3,"; "),REPT(" ",20))</f>
         <v xml:space="preserve">["SAVE_INDEX"] = 2; </v>
       </c>
       <c r="Z3">
@@ -8651,7 +8650,7 @@
         <v>4</v>
       </c>
       <c r="AA3" t="str">
-        <f t="shared" ref="AA3:AA22" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z3)),Z3,"; ")</f>
+        <f t="shared" ref="AA3:AA18" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z3)),Z3,"; ")</f>
         <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB3" t="str">
@@ -8659,31 +8658,31 @@
         <v/>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC22" si="10">IF(NOT(ISBLANK(E3)),CONCATENATE("[""NA""] = ",AB3,"; "),"")</f>
+        <f t="shared" ref="AC3:AC18" si="10">IF(NOT(ISBLANK(E3)),CONCATENATE("[""NA""] = ",AB3,"; "),"")</f>
         <v/>
       </c>
       <c r="AD3" t="str">
-        <f t="shared" ref="AD3:AD22" si="11">TEXT(F3,0)</f>
+        <f t="shared" ref="AD3:AD18" si="11">TEXT(F3,0)</f>
         <v>0</v>
       </c>
       <c r="AE3" t="str">
-        <f t="shared" ref="AE3:AE22" si="12">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD3)),TEXT(AD3,"0"),"; ")</f>
+        <f t="shared" ref="AE3:AE18" si="12">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD3)),TEXT(AD3,"0"),"; ")</f>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF3" t="str">
-        <f t="shared" ref="AF3:AF22" si="13">TEXT(H3,0)</f>
+        <f t="shared" ref="AF3:AF18" si="13">TEXT(H3,0)</f>
         <v>0</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG22" si="14">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF3)),TEXT(AF3,"0"),"; ")</f>
+        <f t="shared" ref="AG3:AG18" si="14">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF3)),TEXT(AF3,"0"),"; ")</f>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH3" t="str">
-        <f t="shared" ref="AH3:AH22" si="15">TEXT(I3,0)</f>
+        <f t="shared" ref="AH3:AH18" si="15">TEXT(I3,0)</f>
         <v>0</v>
       </c>
       <c r="AI3" t="str">
-        <f t="shared" ref="AI3:AI22" si="16">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH3)),TEXT(AH3,"0"),"; ")</f>
+        <f t="shared" ref="AI3:AI18" si="16">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH3)),TEXT(AH3,"0"),"; ")</f>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ3">
@@ -8691,35 +8690,35 @@
         <v>1</v>
       </c>
       <c r="AK3" t="str">
-        <f t="shared" ref="AK3:AK22" si="17">CONCATENATE("[""FACTION""] = ",TEXT(AJ3,"0"),"; ")</f>
+        <f t="shared" ref="AK3:AK18" si="17">CONCATENATE("[""FACTION""] = ",TEXT(AJ3,"0"),"; ")</f>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL3" t="str">
-        <f t="shared" ref="AL3:AL22" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
+        <f t="shared" ref="AL3:AL18" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM3" t="str">
-        <f t="shared" ref="AM3:AM22" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"")</f>
+        <f t="shared" ref="AM3:AM18" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"")</f>
         <v xml:space="preserve">["MIN_LVL"] = "50"; </v>
       </c>
       <c r="AN3" t="str">
-        <f t="shared" ref="AN3:AN22" si="20">IF(LEN(O3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O3)),"""",O3,"""; "),"")</f>
+        <f t="shared" ref="AN3:AN18" si="20">IF(LEN(O3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O3)),"""",O3,"""; "),"")</f>
         <v/>
       </c>
       <c r="AO3" t="str">
-        <f t="shared" ref="AO3:AO22" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
+        <f t="shared" ref="AO3:AO18" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
         <v xml:space="preserve">["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; </v>
       </c>
       <c r="AP3" t="str">
-        <f t="shared" ref="AP3:AP22" si="22">CONCATENATE("[""LORE""] = { [""EN""] = """,L3,"""; }; ")</f>
+        <f t="shared" ref="AP3:AP18" si="22">CONCATENATE("[""LORE""] = { [""EN""] = """,L3,"""; }; ")</f>
         <v xml:space="preserve">["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; </v>
       </c>
       <c r="AQ3" t="str">
-        <f t="shared" ref="AQ3:AQ22" si="23">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K3,"""; }; ")</f>
+        <f t="shared" ref="AQ3:AQ18" si="23">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K3,"""; }; ")</f>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; </v>
       </c>
       <c r="AR3" t="str">
-        <f t="shared" ref="AR3:AR22" si="24">IF(LEN(G3)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G3,"""; }; "),"")</f>
+        <f t="shared" ref="AR3:AR18" si="24">IF(LEN(G3)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G3,"""; }; "),"")</f>
         <v xml:space="preserve">["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; </v>
       </c>
       <c r="AS3" t="str">
@@ -9004,8 +9003,8 @@
       </c>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="C6" s="4" t="s">
-        <v>198</v>
+      <c r="C6" s="3" t="s">
+        <v>205</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>29</v>
@@ -9015,11 +9014,11 @@
       </c>
       <c r="R6" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  [5] = {["CAT_ID"] = 308; }; -- - Monster Player Reward Season 1 -</v>
+        <v xml:space="preserve">  [5] = {["CAT_ID"] = 308; }; -- - Season 1: Strife -</v>
       </c>
       <c r="S6" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [5] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Monster Player Reward Season 1 -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve">  [5] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 1: Strife -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T6">
         <f t="shared" si="3"/>
@@ -9107,7 +9106,7 @@
       </c>
       <c r="AO6" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Monster Player Reward Season 1 -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 1: Strife -"; }; </v>
       </c>
       <c r="AP6" t="str">
         <f t="shared" si="22"/>
@@ -9137,7 +9136,7 @@
         <v>154</v>
       </c>
       <c r="E7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N7" s="2"/>
       <c r="R7" t="str">
@@ -9264,7 +9263,7 @@
         <v>154</v>
       </c>
       <c r="E8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N8" s="2"/>
       <c r="R8" t="str">
@@ -9391,7 +9390,7 @@
         <v>154</v>
       </c>
       <c r="E9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N9" s="2"/>
       <c r="R9" t="str">
@@ -9512,13 +9511,13 @@
         <v>1879490393</v>
       </c>
       <c r="C10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D10" t="s">
         <v>154</v>
       </c>
       <c r="E10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N10" s="2"/>
       <c r="R10" t="str">
@@ -9636,7 +9635,7 @@
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.25">
       <c r="C11" s="3" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>29</v>
@@ -9647,11 +9646,11 @@
       </c>
       <c r="R11" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [10] = {["CAT_ID"] = 327; }; -- - Season of the Nemesis -</v>
+        <v xml:space="preserve"> [10] = {["CAT_ID"] = 327; }; -- - Season 2: Nemesis -</v>
       </c>
       <c r="S11" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [10] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season of the Nemesis -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve"> [10] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 2: Nemesis -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T11">
         <f t="shared" si="3"/>
@@ -9739,7 +9738,7 @@
       </c>
       <c r="AO11" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season of the Nemesis -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 2: Nemesis -"; }; </v>
       </c>
       <c r="AP11" t="str">
         <f t="shared" si="22"/>
@@ -9763,7 +9762,7 @@
         <v>1879509060</v>
       </c>
       <c r="C12" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D12" t="s">
         <v>154</v>
@@ -9884,7 +9883,7 @@
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.25">
       <c r="C13" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>29</v>
@@ -9895,11 +9894,11 @@
       </c>
       <c r="R13" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [12] = {["CAT_ID"] = 328; }; -- - Season of Malice -</v>
+        <v xml:space="preserve"> [12] = {["CAT_ID"] = 328; }; -- - Season 3: Malice -</v>
       </c>
       <c r="S13" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [12] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season of Malice -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve"> [12] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 3: Malice -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T13">
         <f t="shared" si="3"/>
@@ -9987,7 +9986,7 @@
       </c>
       <c r="AO13" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season of Malice -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 3: Malice -"; }; </v>
       </c>
       <c r="AP13" t="str">
         <f t="shared" si="22"/>
@@ -10011,7 +10010,7 @@
         <v>1879509057</v>
       </c>
       <c r="C14" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D14" t="s">
         <v>154</v>
@@ -10132,7 +10131,7 @@
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
       <c r="C15" s="3" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>29</v>
@@ -10143,11 +10142,11 @@
       </c>
       <c r="R15" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [14] = {["CAT_ID"] = 329; }; -- - Season of Scorn -</v>
+        <v xml:space="preserve"> [14] = {["CAT_ID"] = 329; }; -- - Season 4: Scorn -</v>
       </c>
       <c r="S15" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [14] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season of Scorn -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve"> [14] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 4: Scorn -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T15">
         <f t="shared" si="3"/>
@@ -10235,7 +10234,7 @@
       </c>
       <c r="AO15" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season of Scorn -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 4: Scorn -"; }; </v>
       </c>
       <c r="AP15" t="str">
         <f t="shared" si="22"/>
@@ -10259,7 +10258,7 @@
         <v>1879509058</v>
       </c>
       <c r="C16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D16" t="s">
         <v>154</v>
@@ -10380,7 +10379,7 @@
     </row>
     <row r="17" spans="1:45" x14ac:dyDescent="0.25">
       <c r="C17" s="3" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>29</v>
@@ -10391,11 +10390,11 @@
       </c>
       <c r="R17" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [16] = {["CAT_ID"] = 330; }; -- - Season of Spirit -</v>
+        <v xml:space="preserve"> [16] = {["CAT_ID"] = 330; }; -- - Season 5: Spirits -</v>
       </c>
       <c r="S17" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [16] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season of Spirit -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve"> [16] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 5: Spirits -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T17">
         <f t="shared" si="3"/>
@@ -10483,7 +10482,7 @@
       </c>
       <c r="AO17" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season of Spirit -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 5: Spirits -"; }; </v>
       </c>
       <c r="AP17" t="str">
         <f t="shared" si="22"/>
@@ -10507,7 +10506,7 @@
         <v>1879509059</v>
       </c>
       <c r="C18" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D18" t="s">
         <v>154</v>
@@ -10639,11 +10638,11 @@
       </c>
       <c r="R19" t="str">
         <f t="shared" ref="R19:R22" si="26">CONCATENATE(U19,W19,X19,AS19," -- ",C19)</f>
-        <v xml:space="preserve"> [18] = {["CAT_ID"] = 342; }; -- - Monster Player Reward Season 6 -</v>
+        <v xml:space="preserve"> [18] = {["CAT_ID"] = 342; }; -- - Season 6: Rivals -</v>
       </c>
       <c r="S19" s="1" t="str">
         <f t="shared" ref="S19:S22" si="27">CONCATENATE(U19,V19,Y19,AA19,AC19,AE19,AG19,AI19,AK19,AL19,AM19,AN19,AO19,AP19,AQ19,AR19,AS19)</f>
-        <v xml:space="preserve"> [18] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Monster Player Reward Season 6 -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+        <v xml:space="preserve"> [18] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 6: Rivals -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T19">
         <f t="shared" si="3"/>
@@ -10731,7 +10730,7 @@
       </c>
       <c r="AO19" t="str">
         <f t="shared" ref="AO19:AO22" si="45">CONCATENATE("[""NAME""] = { [""EN""] = """,C19,"""; }; ")</f>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Monster Player Reward Season 6 -"; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 6: Rivals -"; }; </v>
       </c>
       <c r="AP19" t="str">
         <f t="shared" ref="AP19:AP22" si="46">CONCATENATE("[""LORE""] = { [""EN""] = """,L19,"""; }; ")</f>
@@ -10755,7 +10754,7 @@
         <v>1879523597</v>
       </c>
       <c r="C20" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D20" t="s">
         <v>154</v>

</xml_diff>

<commit_message>
Added Sea-side Sensation (U48.2) and Frame: Season of Destruction Frame (U48.3), plus other updates.
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-4-The War.xlsx
+++ b/_SourceFiles/DeedInfo-4-The War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD345887-F509-4311-A102-B64DB99E36BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02611CA2-B28A-4C02-A02B-361F40D261F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8205" yWindow="5415" windowWidth="20895" windowHeight="10320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="540" yWindow="480" windowWidth="17295" windowHeight="14430" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="213">
   <si>
     <t>Save Index</t>
   </si>
@@ -672,6 +672,12 @@
   </si>
   <si>
     <t>- Season 6: Rivals -</t>
+  </si>
+  <si>
+    <t>Frame: Season of Destruction Frame</t>
+  </si>
+  <si>
+    <t>- Season 7: Destruction -</t>
   </si>
 </sst>
 </file>
@@ -8614,35 +8620,35 @@
         <v>50</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R18" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
+        <f t="shared" ref="R3:R24" si="1">CONCATENATE(U3,W3,X3,AS3," -- ",C3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879071836; }; -- Conquest of Dargazag</v>
       </c>
       <c r="S3" s="1" t="str">
-        <f t="shared" ref="S3:S18" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
+        <f t="shared" ref="S3:S24" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
         <v xml:space="preserve">  [2] = {["ID"] = 1879071836; ["SAVE_INDEX"] = 2; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; ["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; };</v>
       </c>
       <c r="T3">
-        <f t="shared" ref="T3:T22" si="3">ROW()-1</f>
+        <f t="shared" ref="T3:T24" si="3">ROW()-1</f>
         <v>2</v>
       </c>
       <c r="U3" t="str">
-        <f t="shared" ref="U3:U18" si="4">CONCATENATE(REPT(" ",3-LEN(T3)),"[",T3,"] = {")</f>
+        <f t="shared" ref="U3:U24" si="4">CONCATENATE(REPT(" ",3-LEN(T3)),"[",T3,"] = {")</f>
         <v xml:space="preserve">  [2] = {</v>
       </c>
       <c r="V3" t="str">
-        <f t="shared" ref="V3:V18" si="5">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"                     ")</f>
+        <f t="shared" ref="V3:V24" si="5">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"                     ")</f>
         <v xml:space="preserve">["ID"] = 1879071836; </v>
       </c>
       <c r="W3" t="str">
-        <f t="shared" ref="W3:W18" si="6">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
+        <f t="shared" ref="W3:W24" si="6">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879071836; </v>
       </c>
       <c r="X3" t="str">
-        <f t="shared" ref="X3:X18" si="7">IF(LEN(P3)&gt;0,CONCATENATE("[""CAT_ID""] = ",P3,"; "),"")</f>
+        <f t="shared" ref="X3:X24" si="7">IF(LEN(P3)&gt;0,CONCATENATE("[""CAT_ID""] = ",P3,"; "),"")</f>
         <v/>
       </c>
       <c r="Y3" s="1" t="str">
-        <f t="shared" ref="Y3:Y18" si="8">IF(LEN(B3)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B3)),B3,"; "),REPT(" ",20))</f>
+        <f t="shared" ref="Y3:Y24" si="8">IF(LEN(B3)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B3)),B3,"; "),REPT(" ",20))</f>
         <v xml:space="preserve">["SAVE_INDEX"] = 2; </v>
       </c>
       <c r="Z3">
@@ -8650,7 +8656,7 @@
         <v>4</v>
       </c>
       <c r="AA3" t="str">
-        <f t="shared" ref="AA3:AA18" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z3)),Z3,"; ")</f>
+        <f t="shared" ref="AA3:AA24" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z3)),Z3,"; ")</f>
         <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB3" t="str">
@@ -8658,31 +8664,31 @@
         <v/>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC18" si="10">IF(NOT(ISBLANK(E3)),CONCATENATE("[""NA""] = ",AB3,"; "),"")</f>
+        <f t="shared" ref="AC3:AC24" si="10">IF(NOT(ISBLANK(E3)),CONCATENATE("[""NA""] = ",AB3,"; "),"")</f>
         <v/>
       </c>
       <c r="AD3" t="str">
-        <f t="shared" ref="AD3:AD18" si="11">TEXT(F3,0)</f>
+        <f t="shared" ref="AD3:AD24" si="11">TEXT(F3,0)</f>
         <v>0</v>
       </c>
       <c r="AE3" t="str">
-        <f t="shared" ref="AE3:AE18" si="12">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD3)),TEXT(AD3,"0"),"; ")</f>
+        <f t="shared" ref="AE3:AE24" si="12">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD3)),TEXT(AD3,"0"),"; ")</f>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF3" t="str">
-        <f t="shared" ref="AF3:AF18" si="13">TEXT(H3,0)</f>
+        <f t="shared" ref="AF3:AF24" si="13">TEXT(H3,0)</f>
         <v>0</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG18" si="14">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF3)),TEXT(AF3,"0"),"; ")</f>
+        <f t="shared" ref="AG3:AG24" si="14">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF3)),TEXT(AF3,"0"),"; ")</f>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH3" t="str">
-        <f t="shared" ref="AH3:AH18" si="15">TEXT(I3,0)</f>
+        <f t="shared" ref="AH3:AH24" si="15">TEXT(I3,0)</f>
         <v>0</v>
       </c>
       <c r="AI3" t="str">
-        <f t="shared" ref="AI3:AI18" si="16">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH3)),TEXT(AH3,"0"),"; ")</f>
+        <f t="shared" ref="AI3:AI24" si="16">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH3)),TEXT(AH3,"0"),"; ")</f>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ3">
@@ -8690,39 +8696,39 @@
         <v>1</v>
       </c>
       <c r="AK3" t="str">
-        <f t="shared" ref="AK3:AK18" si="17">CONCATENATE("[""FACTION""] = ",TEXT(AJ3,"0"),"; ")</f>
+        <f t="shared" ref="AK3:AK24" si="17">CONCATENATE("[""FACTION""] = ",TEXT(AJ3,"0"),"; ")</f>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL3" t="str">
-        <f t="shared" ref="AL3:AL18" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
+        <f t="shared" ref="AL3:AL24" si="18">CONCATENATE("[""TIER""] = ",TEXT(M3,"0"),"; ")</f>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM3" t="str">
-        <f t="shared" ref="AM3:AM18" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"")</f>
+        <f t="shared" ref="AM3:AM24" si="19">IF(LEN(N3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N3)),"""",N3,"""; "),"")</f>
         <v xml:space="preserve">["MIN_LVL"] = "50"; </v>
       </c>
       <c r="AN3" t="str">
-        <f t="shared" ref="AN3:AN18" si="20">IF(LEN(O3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O3)),"""",O3,"""; "),"")</f>
+        <f t="shared" ref="AN3:AN24" si="20">IF(LEN(O3)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O3)),"""",O3,"""; "),"")</f>
         <v/>
       </c>
       <c r="AO3" t="str">
-        <f t="shared" ref="AO3:AO18" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
+        <f t="shared" ref="AO3:AO24" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
         <v xml:space="preserve">["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; </v>
       </c>
       <c r="AP3" t="str">
-        <f t="shared" ref="AP3:AP18" si="22">CONCATENATE("[""LORE""] = { [""EN""] = """,L3,"""; }; ")</f>
+        <f t="shared" ref="AP3:AP24" si="22">CONCATENATE("[""LORE""] = { [""EN""] = """,L3,"""; }; ")</f>
         <v xml:space="preserve">["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; </v>
       </c>
       <c r="AQ3" t="str">
-        <f t="shared" ref="AQ3:AQ18" si="23">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K3,"""; }; ")</f>
+        <f t="shared" ref="AQ3:AQ24" si="23">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K3,"""; }; ")</f>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; </v>
       </c>
       <c r="AR3" t="str">
-        <f t="shared" ref="AR3:AR18" si="24">IF(LEN(G3)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G3,"""; }; "),"")</f>
+        <f t="shared" ref="AR3:AR24" si="24">IF(LEN(G3)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G3,"""; }; "),"")</f>
         <v xml:space="preserve">["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; </v>
       </c>
       <c r="AS3" t="str">
-        <f t="shared" ref="AS3:AS22" si="25">CONCATENATE("};")</f>
+        <f t="shared" ref="AS3:AS24" si="25">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
@@ -10637,11 +10643,11 @@
         <v>342</v>
       </c>
       <c r="R19" t="str">
-        <f t="shared" ref="R19:R22" si="26">CONCATENATE(U19,W19,X19,AS19," -- ",C19)</f>
+        <f t="shared" si="1"/>
         <v xml:space="preserve"> [18] = {["CAT_ID"] = 342; }; -- - Season 6: Rivals -</v>
       </c>
       <c r="S19" s="1" t="str">
-        <f t="shared" ref="S19:S22" si="27">CONCATENATE(U19,V19,Y19,AA19,AC19,AE19,AG19,AI19,AK19,AL19,AM19,AN19,AO19,AP19,AQ19,AR19,AS19)</f>
+        <f t="shared" si="2"/>
         <v xml:space="preserve"> [18] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 6: Rivals -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T19">
@@ -10649,23 +10655,23 @@
         <v>18</v>
       </c>
       <c r="U19" t="str">
-        <f t="shared" ref="U19:U22" si="28">CONCATENATE(REPT(" ",3-LEN(T19)),"[",T19,"] = {")</f>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> [18] = {</v>
       </c>
       <c r="V19" t="str">
-        <f t="shared" ref="V19:V22" si="29">IF(LEN(A19)&gt;0,CONCATENATE("[""ID""] = ",A19,"; "),"                     ")</f>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">                     </v>
       </c>
       <c r="W19" t="str">
-        <f t="shared" ref="W19:W22" si="30">IF(LEN(A19)&gt;0,CONCATENATE("[""ID""] = ",A19,"; "),"")</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="X19" t="str">
-        <f t="shared" ref="X19:X22" si="31">IF(LEN(P19)&gt;0,CONCATENATE("[""CAT_ID""] = ",P19,"; "),"")</f>
+        <f t="shared" si="7"/>
         <v xml:space="preserve">["CAT_ID"] = 342; </v>
       </c>
       <c r="Y19" s="1" t="str">
-        <f t="shared" ref="Y19:Y22" si="32">IF(LEN(B19)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B19)),B19,"; "),REPT(" ",20))</f>
+        <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
       <c r="Z19">
@@ -10673,7 +10679,7 @@
         <v>14</v>
       </c>
       <c r="AA19" t="str">
-        <f t="shared" ref="AA19:AA22" si="33">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z19)),Z19,"; ")</f>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">["TYPE"] = 14; </v>
       </c>
       <c r="AB19" t="str">
@@ -10681,31 +10687,31 @@
         <v/>
       </c>
       <c r="AC19" t="str">
-        <f t="shared" ref="AC19:AC22" si="34">IF(NOT(ISBLANK(E19)),CONCATENATE("[""NA""] = ",AB19,"; "),"")</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AD19" t="str">
-        <f t="shared" ref="AD19:AD22" si="35">TEXT(F19,0)</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AE19" t="str">
-        <f t="shared" ref="AE19:AE22" si="36">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD19)),TEXT(AD19,"0"),"; ")</f>
+        <f t="shared" si="12"/>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF19" t="str">
-        <f t="shared" ref="AF19:AF22" si="37">TEXT(H19,0)</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG19" t="str">
-        <f t="shared" ref="AG19:AG22" si="38">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF19)),TEXT(AF19,"0"),"; ")</f>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH19" t="str">
-        <f t="shared" ref="AH19:AH22" si="39">TEXT(I19,0)</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AI19" t="str">
-        <f t="shared" ref="AI19:AI22" si="40">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH19)),TEXT(AH19,"0"),"; ")</f>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ19">
@@ -10713,35 +10719,35 @@
         <v>1</v>
       </c>
       <c r="AK19" t="str">
-        <f t="shared" ref="AK19:AK22" si="41">CONCATENATE("[""FACTION""] = ",TEXT(AJ19,"0"),"; ")</f>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL19" t="str">
-        <f t="shared" ref="AL19:AL22" si="42">CONCATENATE("[""TIER""] = ",TEXT(M19,"0"),"; ")</f>
+        <f t="shared" si="18"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM19" t="str">
-        <f t="shared" ref="AM19:AM22" si="43">IF(LEN(N19)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N19)),"""",N19,"""; "),"")</f>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="AN19" t="str">
-        <f t="shared" ref="AN19:AN22" si="44">IF(LEN(O19)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O19)),"""",O19,"""; "),"")</f>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="AO19" t="str">
-        <f t="shared" ref="AO19:AO22" si="45">CONCATENATE("[""NAME""] = { [""EN""] = """,C19,"""; }; ")</f>
+        <f t="shared" si="21"/>
         <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 6: Rivals -"; }; </v>
       </c>
       <c r="AP19" t="str">
-        <f t="shared" ref="AP19:AP22" si="46">CONCATENATE("[""LORE""] = { [""EN""] = """,L19,"""; }; ")</f>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AQ19" t="str">
-        <f t="shared" ref="AQ19:AQ22" si="47">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K19,"""; }; ")</f>
+        <f t="shared" si="23"/>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AR19" t="str">
-        <f t="shared" ref="AR19:AR22" si="48">IF(LEN(G19)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G19,"""; }; "),"")</f>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="AS19" t="str">
@@ -10761,11 +10767,11 @@
       </c>
       <c r="N20" s="2"/>
       <c r="R20" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="1"/>
         <v xml:space="preserve"> [19] = {["ID"] = 1879523597; }; -- Title: Bastion of Light</v>
       </c>
       <c r="S20" s="1" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="2"/>
         <v xml:space="preserve"> [19] = {["ID"] = 1879523597;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Bastion of Light"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T20">
@@ -10773,23 +10779,23 @@
         <v>19</v>
       </c>
       <c r="U20" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> [19] = {</v>
       </c>
       <c r="V20" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">["ID"] = 1879523597; </v>
       </c>
       <c r="W20" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve">["ID"] = 1879523597; </v>
       </c>
       <c r="X20" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="Y20" s="1" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
       <c r="Z20">
@@ -10797,7 +10803,7 @@
         <v>7</v>
       </c>
       <c r="AA20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">["TYPE"] =  7; </v>
       </c>
       <c r="AB20" t="str">
@@ -10805,31 +10811,31 @@
         <v/>
       </c>
       <c r="AC20" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AD20" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AE20" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="12"/>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF20" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG20" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH20" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AI20" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ20">
@@ -10837,35 +10843,35 @@
         <v>1</v>
       </c>
       <c r="AK20" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL20" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="18"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM20" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="AN20" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="AO20" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="21"/>
         <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Bastion of Light"; }; </v>
       </c>
       <c r="AP20" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AQ20" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" si="23"/>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AR20" t="str">
-        <f t="shared" si="48"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="AS20" t="str">
@@ -10874,78 +10880,86 @@
       </c>
     </row>
     <row r="21" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D21" s="2"/>
+      <c r="C21" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="N21" s="2"/>
+      <c r="P21">
+        <v>349</v>
+      </c>
       <c r="R21" t="str">
-        <f t="shared" si="26"/>
-        <v xml:space="preserve"> [20] = {}; -- </v>
-      </c>
-      <c r="S21" s="1" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> [20] = {["CAT_ID"] = 349; }; -- - Season 7: Destruction -</v>
+      </c>
+      <c r="S21" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [20] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 7: Destruction -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T21">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="U21" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> [20] = {</v>
       </c>
       <c r="V21" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">                     </v>
       </c>
       <c r="W21" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="X21" t="str">
-        <f t="shared" si="31"/>
-        <v/>
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">["CAT_ID"] = 349; </v>
       </c>
       <c r="Y21" s="1" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
-      <c r="Z21" t="e">
+      <c r="Z21">
         <f>VLOOKUP(D21,[1]Type!A$2:B$18,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AA21" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <v>14</v>
+      </c>
+      <c r="AA21" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] = 14; </v>
       </c>
       <c r="AB21" t="str">
         <f>IF(NOT(ISBLANK(E21)),VLOOKUP(E21,[1]Type!D$2:E$6,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="AC21" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AD21" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AE21" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="12"/>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF21" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG21" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH21" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AI21" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ21">
@@ -10953,35 +10967,35 @@
         <v>1</v>
       </c>
       <c r="AK21" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL21" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="18"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM21" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="AN21" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="AO21" t="str">
-        <f t="shared" si="45"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+        <f t="shared" si="21"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 7: Destruction -"; }; </v>
       </c>
       <c r="AP21" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AQ21" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" si="23"/>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AR21" t="str">
-        <f t="shared" si="48"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="AS21" t="str">
@@ -10990,78 +11004,86 @@
       </c>
     </row>
     <row r="22" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D22" s="2"/>
+      <c r="A22">
+        <v>1879526227</v>
+      </c>
+      <c r="C22" t="s">
+        <v>211</v>
+      </c>
+      <c r="D22" t="s">
+        <v>154</v>
+      </c>
       <c r="N22" s="2"/>
       <c r="R22" t="str">
-        <f t="shared" si="26"/>
-        <v xml:space="preserve"> [21] = {}; -- </v>
-      </c>
-      <c r="S22" s="1" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> [21] = {["ID"] = 1879526227; }; -- Frame: Season of Destruction Frame</v>
+      </c>
+      <c r="S22" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [21] = {["ID"] = 1879526227;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Frame: Season of Destruction Frame"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T22">
         <f t="shared" si="3"/>
         <v>21</v>
       </c>
       <c r="U22" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> [21] = {</v>
       </c>
       <c r="V22" t="str">
-        <f t="shared" si="29"/>
-        <v xml:space="preserve">                     </v>
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["ID"] = 1879526227; </v>
       </c>
       <c r="W22" t="str">
-        <f t="shared" si="30"/>
-        <v/>
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">["ID"] = 1879526227; </v>
       </c>
       <c r="X22" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="Y22" s="1" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
-      <c r="Z22" t="e">
+      <c r="Z22">
         <f>VLOOKUP(D22,[1]Type!A$2:B$18,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AA22" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <v>7</v>
+      </c>
+      <c r="AA22" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
       </c>
       <c r="AB22" t="str">
         <f>IF(NOT(ISBLANK(E22)),VLOOKUP(E22,[1]Type!D$2:E$6,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="AC22" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="AD22" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AE22" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="12"/>
         <v xml:space="preserve">["VXP"] = 0; </v>
       </c>
       <c r="AF22" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG22" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["LP"] = 0; </v>
       </c>
       <c r="AH22" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AI22" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">["REP"] = 0; </v>
       </c>
       <c r="AJ22">
@@ -11069,35 +11091,35 @@
         <v>1</v>
       </c>
       <c r="AK22" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">["FACTION"] = 1; </v>
       </c>
       <c r="AL22" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="18"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="AM22" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="AN22" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="AO22" t="str">
-        <f t="shared" si="45"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+        <f t="shared" si="21"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Frame: Season of Destruction Frame"; }; </v>
       </c>
       <c r="AP22" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AQ22" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" si="23"/>
         <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
       </c>
       <c r="AR22" t="str">
-        <f t="shared" si="48"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="AS22" t="str">
@@ -11108,13 +11130,233 @@
     <row r="23" spans="1:45" x14ac:dyDescent="0.25">
       <c r="D23" s="2"/>
       <c r="N23" s="2"/>
-      <c r="S23" s="1"/>
-      <c r="Y23" s="1"/>
+      <c r="R23" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> [22] = {}; -- </v>
+      </c>
+      <c r="S23" s="1" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="3"/>
+        <v>22</v>
+      </c>
+      <c r="U23" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> [22] = {</v>
+      </c>
+      <c r="V23" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W23" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="Y23" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z23" t="e">
+        <f>VLOOKUP(D23,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA23" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB23" t="str">
+        <f>IF(NOT(ISBLANK(E23)),VLOOKUP(E23,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC23" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="AD23" t="str">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AE23" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF23" t="str">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AG23" t="str">
+        <f t="shared" si="14"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH23" t="str">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AI23" t="str">
+        <f t="shared" si="16"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ23">
+        <f>IF(NOT(ISBLANK(J23)),VLOOKUP(J23,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK23" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL23" t="str">
+        <f t="shared" si="18"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM23" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="AN23" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="AO23" t="str">
+        <f t="shared" si="21"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP23" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ23" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR23" t="str">
+        <f t="shared" si="24"/>
+        <v/>
+      </c>
+      <c r="AS23" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="24" spans="1:45" x14ac:dyDescent="0.25">
       <c r="N24" s="2"/>
-      <c r="S24" s="1"/>
-      <c r="Y24" s="1"/>
+      <c r="R24" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> [23] = {}; -- </v>
+      </c>
+      <c r="S24" s="1" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="U24" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> [23] = {</v>
+      </c>
+      <c r="V24" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W24" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="Y24" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z24" t="e">
+        <f>VLOOKUP(D24,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA24" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB24" t="str">
+        <f>IF(NOT(ISBLANK(E24)),VLOOKUP(E24,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC24" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="AD24" t="str">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AE24" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF24" t="str">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AG24" t="str">
+        <f t="shared" si="14"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH24" t="str">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AI24" t="str">
+        <f t="shared" si="16"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ24">
+        <f>IF(NOT(ISBLANK(J24)),VLOOKUP(J24,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK24" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL24" t="str">
+        <f t="shared" si="18"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM24" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="AN24" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="AO24" t="str">
+        <f t="shared" si="21"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP24" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ24" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR24" t="str">
+        <f t="shared" si="24"/>
+        <v/>
+      </c>
+      <c r="AS24" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="25" spans="1:45" x14ac:dyDescent="0.25">
       <c r="S25" s="1"/>

</xml_diff>